<commit_message>
Mise à jour du referenceRange des profils cholestérol (#138)
* suppression des contraintes sur le referencerange

* update refrange e26eb5a9f1cf704b9e832eb55123fa2133969c16
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-observation-cholesterol-hdl.xlsx
+++ b/main/ig/StructureDefinition-mesures-observation-cholesterol-hdl.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-18T17:41:07+00:00</t>
+    <t>2026-03-31T09:00:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1713,7 +1713,7 @@
     <t>Observation.referenceRange.type</t>
   </si>
   <si>
-    <t>Reference range qualifier</t>
+    <t>Le type de référence permet d'indiquer s'il s'agit d'un intervalle de réfence ou d'un objectif cible.</t>
   </si>
   <si>
     <t>Codes to indicate the what part of the targeted reference population it applies to. For example, the normal or therapeutic range.</t>
@@ -9888,7 +9888,7 @@
       </c>
       <c r="E64" s="2"/>
       <c r="F64" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="G64" t="s" s="2">
         <v>93</v>
@@ -10009,7 +10009,7 @@
         <v>80</v>
       </c>
       <c r="G65" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="H65" t="s" s="2">
         <v>82</v>
@@ -10127,7 +10127,7 @@
         <v>80</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="H66" t="s" s="2">
         <v>82</v>

</xml_diff>